<commit_message>
US-first: AI for Your Business, One-Person AI, Etsy, Dropshipping (+ new worksheets), POD, Reselling, TikTok; every page en-US
</commit_message>
<xml_diff>
--- a/resources/ai-for-your-business/files/aifyb-adv-commercial-test.xlsx
+++ b/resources/ai-for-your-business/files/aifyb-adv-commercial-test.xlsx
@@ -20,8 +20,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="£#,##0"/>
-    <numFmt numFmtId="166" formatCode="£#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="$#,##0"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="8">
@@ -595,7 +595,7 @@
       <c r="B11" s="4" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>a labelled trial rate is fine; a quiet discount is not</t>
+          <t>a labeled trial rate is fine; a quiet discount is not</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -696,7 +696,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>The controlled commercial test</t>
+          <t>The commercial probe</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>⚠️ The unit that matters is realised margin PER DELIVERY HOUR — price alone tells you</t>
+          <t>⚠️ The unit that matters is realized margin PER DELIVERY HOUR — price alone tells you</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Revenue over the term (£)</t>
+          <t>Revenue over the term ($)</t>
         </is>
       </c>
       <c r="B11" s="4" t="n"/>
@@ -795,7 +795,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Direct delivery cost over the term (£)</t>
+          <t>Direct delivery cost over the term ($)</t>
         </is>
       </c>
       <c r="B12" s="4" t="n"/>
@@ -834,250 +834,264 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Term length (months)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n"/>
+      <c r="C15" s="4" t="n"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>the term you declared, 1-3 months</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>CALCULATED</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Acceptance rate</t>
-        </is>
-      </c>
-      <c r="B17" s="7">
-        <f>IF(OR(COUNT(B9)=0,COUNT(B10)=0,B9=0),"—",B10/B9)</f>
-        <v/>
-      </c>
-      <c r="C17" s="7">
-        <f>IF(OR(COUNT(C9)=0,COUNT(C10)=0,C9=0),"—",C10/C9)</f>
-        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Realised margin (£)</t>
-        </is>
-      </c>
-      <c r="B18" s="8">
-        <f>IF(COUNT(B11)*COUNT(B12)=0,"—",B11-B12)</f>
-        <v/>
-      </c>
-      <c r="C18" s="8">
-        <f>IF(COUNT(C11)*COUNT(C12)=0,"—",C11-C12)</f>
+          <t>Acceptance rate</t>
+        </is>
+      </c>
+      <c r="B18" s="7">
+        <f>IF(OR(COUNT(B9)=0,COUNT(B10)=0,B9=0),"—",B10/B9)</f>
+        <v/>
+      </c>
+      <c r="C18" s="7">
+        <f>IF(OR(COUNT(C9)=0,COUNT(C10)=0,C9=0),"—",C10/C9)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Margin per delivery hour (£)</t>
-        </is>
-      </c>
-      <c r="B19" s="9">
-        <f>IF(OR(COUNT(B11)=0,COUNT(B12)=0,COUNT(B13)=0,B13=0),"—",(B11-B12)/B13)</f>
-        <v/>
-      </c>
-      <c r="C19" s="9">
-        <f>IF(OR(COUNT(C11)=0,COUNT(C12)=0,COUNT(C13)=0,C13=0),"—",(C11-C12)/C13)</f>
+          <t>Realized margin ($)</t>
+        </is>
+      </c>
+      <c r="B19" s="8">
+        <f>IF(COUNT(B11)*COUNT(B12)=0,"—",B11-B12)</f>
+        <v/>
+      </c>
+      <c r="C19" s="8">
+        <f>IF(COUNT(C11)*COUNT(C12)=0,"—",C11-C12)</f>
         <v/>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Burden: hours per client</t>
-        </is>
-      </c>
-      <c r="B20" s="10">
-        <f>IF(OR(COUNT(B13)=0,COUNT(B10)=0,B10=0),"—",B13/B10)</f>
-        <v/>
-      </c>
-      <c r="C20" s="10">
-        <f>IF(OR(COUNT(C13)=0,COUNT(C10)=0,C10=0),"—",C13/C10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="6" t="inlineStr">
+          <t>Margin per delivery hour ($)</t>
+        </is>
+      </c>
+      <c r="B20" s="9">
+        <f>IF(OR(COUNT(B11)=0,COUNT(B12)=0,COUNT(B13)=0,B13=0),"—",(B11-B12)/B13)</f>
+        <v/>
+      </c>
+      <c r="C20" s="9">
+        <f>IF(OR(COUNT(C11)=0,COUNT(C12)=0,COUNT(C13)=0,C13=0),"—",(C11-C12)/C13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Burden: hours per client per month</t>
+        </is>
+      </c>
+      <c r="B21" s="10">
+        <f>IF(OR(COUNT(B13)=0,COUNT(B10)=0,B10=0,COUNT(B15)=0,B15=0),"—",B13/B10/B15)</f>
+        <v/>
+      </c>
+      <c r="C21" s="10">
+        <f>IF(OR(COUNT(C13)=0,COUNT(C10)=0,C10=0,COUNT(C15)=0,C15=0),"—",C13/C10/C15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
         <is>
           <t>YOUR DECISION RULE — set these THRESHOLDS before you offer anything</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Numbers, not sentences — so the branch is computed rather than argued. Thresholds come</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>from YOUR baseline economics and capacity; there is no defensible published figure at</t>
+          <t>Numbers, not sentences — so the branch is computed rather than argued. Thresholds come</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>from YOUR baseline economics and capacity; there is no defensible published figure at</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
           <t>this scale. Once these are set, every possible result lands on exactly one branch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>Minimum acceptances to proceed</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="n"/>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>of those offered</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Burden cap (hours per client per month)</t>
+          <t>Minimum acceptances to proceed</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>over this and we narrow</t>
+          <t>of those offered</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>Acceptances below which the package is wrong</t>
+          <t>Burden cap (hours per client per month)</t>
         </is>
       </c>
       <c r="B29" s="4" t="n"/>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>not the price — go back to chapter 4</t>
+          <t>over this and we narrow</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>Can we staff more than the accepted number? (y/n)</t>
+          <t>Acceptances below which the package is wrong</t>
         </is>
       </c>
       <c r="B30" s="4" t="n"/>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>no means CAP</t>
+          <t>not the price — go back to chapter 4</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>Thresholds set on (date)</t>
+          <t>Can we staff more than the accepted number? (y/n)</t>
         </is>
       </c>
       <c r="B31" s="4" t="n"/>
       <c r="D31" s="2" t="inlineStr">
         <is>
+          <t>no means CAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Thresholds set on (date)</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="n"/>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
           <t>before any offer goes out</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>THE BRANCH — computed</t>
         </is>
       </c>
-      <c r="B33" s="11">
-        <f>IF(OR(COUNT(B27)=0,COUNT(B28)=0,COUNT(B29)=0,COUNTA(B30)=0,NOT(ISNUMBER(B31))),"NOT READY - set every threshold, and date the rule with a real date, before you offer anything",IF(B29&gt;B27,"NOT READY - the stop floor cannot be above the minimum to proceed",IF(AND(ISNUMBER(B10),ISNUMBER(B9),B10&gt;B9),"CHECK THE NUMBERS - more accepted than offered. Fix that before reading a branch.",IF(COUNT(B10)=0,"waiting for results",IF(B10&lt;B29,"STOP - the package is wrong, not the price",IF(B10&lt;B27,"NARROW AND RETEST - real interest, wrong shape",IF(OR(NOT(ISNUMBER(B19)),NOT(ISNUMBER(C19))),"NARROW - margin per delivery hour not measurable yet",IF(B19&lt;=C19,"NARROW - margin per delivery hour does not beat the baseline cohort",IF(OR(NOT(ISNUMBER(B20)),B20&gt;B28),"NARROW - burden over the cap; cut scope, same price",IF(LOWER(TRIM(B30))&lt;&gt;"y","CAP - hold the client count, fix the constraint","CONTINUE - becomes the standard offer"))))))))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ Fails closed: a missing threshold, an undated rule or an unmeasurable margin all</t>
-        </is>
+      <c r="B34" s="11">
+        <f>IF(OR(COUNT(B28)=0,COUNT(B29)=0,COUNT(B30)=0,COUNTA(B31)=0,NOT(ISNUMBER(B32))),"NOT READY - set every threshold, and date the rule with a real date, before you offer anything",IF(B30&gt;B28,"NOT READY - the stop floor cannot be above the minimum to proceed",IF(AND(ISNUMBER(B10),ISNUMBER(B9),B10&gt;B9),"CHECK THE NUMBERS - more accepted than offered. Fix that before reading a branch.",IF(COUNT(B10)=0,"waiting for results",IF(B10&lt;B30,"STOP - the package is wrong, not the price",IF(B10&lt;B28,IF(AND(ISNUMBER(B20),ISNUMBER(C20),ISNUMBER(B21)),IF(AND(B20&gt;C20,B21&lt;B29),"NARROW AND RETEST - real interest, wrong shape","STOP - not enough interest to justify fixing: margin or burden fails too"),"NARROW AND RETEST - real interest; measure margin and burden before deciding"),IF(OR(NOT(ISNUMBER(B20)),NOT(ISNUMBER(C20))),"NARROW - margin per delivery hour not measurable yet",IF(B20&lt;=C20,"NARROW - margin per delivery hour does not beat the baseline cohort",IF(OR(NOT(ISNUMBER(B21)),B21&gt;=B29),"NARROW - burden at or over the cap; cut scope, same price",IF(LOWER(TRIM(B31))&lt;&gt;"y","CAP - hold the client count, fix the constraint","CONTINUE - becomes the standard offer"))))))))))</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>⚠️ Fails closed: a missing threshold, an undated rule or an unmeasurable margin all</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
           <t>read as NOT READY or NARROW — never as CONTINUE.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="2" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>Retention is the CONFIRMATION step at first renewal, not part of the first decision.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>⚠️ FAIRNESS AND THE LAW. Offering a genuinely NEW package at a new price, to clients as</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>they renew, is ordinary practice — the thing being bought has changed. Charging similar</t>
+          <t>⚠️ FAIRNESS. Offering a genuinely NEW package at a new price, to clients as</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>clients materially different rates for the IDENTICAL legacy deliverable is where the</t>
+          <t>they renew, is ordinary practice — the thing being bought has changed. Charging similar</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>trouble lives. Write down the commercial basis for cohort assignment before you assign;</t>
+          <t>clients materially different rates for the IDENTICAL legacy deliverable is where the</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>make sure it is not a proxy for any protected characteristic; check existing contracts;</t>
+          <t>trouble lives. Write down the commercial basis for cohort assignment before you assign;</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>be able to explain the difference to any client who asks; check existing contracts;</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
           <t>and put it to your own professional adviser. Not legal advice.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="B9:C14" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Out of range" error="Enter a number between 0 and 1000000." type="decimal" operator="between">
+    <dataValidation sqref="B9:C15" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Out of range" error="Enter a number between 0 and 1000000." type="decimal" operator="between">
       <formula1>0</formula1>
       <formula2>1000000</formula2>
     </dataValidation>
-    <dataValidation sqref="B30" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="y or n" error="Enter y or n. A blank counts as a FAIL, never a pass." type="list">
+    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="y or n" error="Enter y or n. A blank counts as a FAIL, never a pass." type="list">
       <formula1>"y,n"</formula1>
     </dataValidation>
-    <dataValidation sqref="B31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Enter a real date" error="Type a date. 'Soon' and 'later' are not dates, and the gate checks for a real one." type="date" operator="greaterThan">
+    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Enter a real date" error="Type a date. 'Soon' and 'later' are not dates, and the gate checks for a real one." type="date" operator="greaterThan">
       <formula1>DATE(2020,1,1)</formula1>
     </dataValidation>
   </dataValidations>
@@ -1118,7 +1132,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>A written undertaking to a named paying client. 60-90 days minimum. Not irreversible —</t>
+          <t>A written undertaking to a named paying client. Initial term: 60-90 days. Not irreversible —</t>
         </is>
       </c>
     </row>

</xml_diff>